<commit_message>
Python Package for the GUI created
</commit_message>
<xml_diff>
--- a/Documentation/cards.xlsx
+++ b/Documentation/cards.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="120" windowWidth="11490" windowHeight="2625" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="120" windowWidth="11490" windowHeight="2625"/>
   </bookViews>
   <sheets>
     <sheet name="node parameters" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="65">
   <si>
     <t>node</t>
   </si>
@@ -207,6 +207,9 @@
   </si>
   <si>
     <t>outflow</t>
+  </si>
+  <si>
+    <t>Enclosure</t>
   </si>
 </sst>
 </file>
@@ -693,7 +696,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:I19"/>
+  <dimension ref="B2:I20"/>
   <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
@@ -1046,6 +1049,32 @@
       <c r="G19" s="11"/>
       <c r="H19" s="11"/>
       <c r="I19" s="12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" ht="12" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="9">
+        <v>16</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="H20" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="I20" s="12" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>